<commit_message>
Add: end of quest
* Update: ring message, PositionCell rotation to 40
* Fix: letter text cutoff
</commit_message>
<xml_diff>
--- a/Docs/Dialogue.xlsx
+++ b/Docs/Dialogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0B71D6-C43D-4BD9-96AC-A43276E405DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D07548-A2BB-44BE-A308-A85008FF746E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
   <si>
     <t>Character</t>
   </si>
@@ -81,6 +81,9 @@
   <si>
     <t>In all likelyhood I've just said this to you already, but just in case (or you clicked ahead): I love you very much my darling. Aoife, you mean so much to me. Since you have been in my life my heart has been filled with joy and love for you.</t>
   </si>
+  <si>
+    <t>Aah! Wifey! Using the soul gem did the trick too, which I suspected it might. Anyway, thank you for rescuing me!</t>
+  </si>
 </sst>
 </file>
 
@@ -109,7 +112,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -119,6 +122,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -135,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -144,12 +153,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -368,7 +381,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:E1000"/>
+  <dimension ref="B1:E1001"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.109375" customWidth="1"/>
@@ -397,84 +410,92 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="5" t="s">
+    <row r="4" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
+    <row r="8" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>16</v>
+      <c r="C8" s="7" t="s">
+        <v>5</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>17</v>
+      <c r="D8" s="8" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D10" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D10" s="1"/>
-    </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D11" s="1"/>
     </row>
@@ -3444,6 +3465,9 @@
     </row>
     <row r="1000" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D1000" s="1"/>
+    </row>
+    <row r="1001" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1001" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update: additional diolgue for greeting and topics
* Fix: removed debug messages
</commit_message>
<xml_diff>
--- a/Docs/Dialogue.xlsx
+++ b/Docs/Dialogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D07548-A2BB-44BE-A308-A85008FF746E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAAEA50-D3B7-4ECD-9912-9A1469423918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
   <si>
     <t>Character</t>
   </si>
@@ -83,6 +83,66 @@
   </si>
   <si>
     <t>Aah! Wifey! Using the soul gem did the trick too, which I suspected it might. Anyway, thank you for rescuing me!</t>
+  </si>
+  <si>
+    <t>Checks</t>
+  </si>
+  <si>
+    <t>Greeting alt</t>
+  </si>
+  <si>
+    <t>Thank you so much for rescuing me! Honestly I wasn't… wait, I'm completely naked. Sweetie, before you go I'm going to have to take my clothes back.</t>
+  </si>
+  <si>
+    <t>Thank you so much for rescuing me my darling… ah I see that your looting instincts kicked in!</t>
+  </si>
+  <si>
+    <t>Greeting generic</t>
+  </si>
+  <si>
+    <t>Again, thank you so much my darling. You are my sweet moonlight!</t>
+  </si>
+  <si>
+    <t>rescuing me - generic</t>
+  </si>
+  <si>
+    <t>And what a marvelous job you did!</t>
+  </si>
+  <si>
+    <t>And what a marvelous job you did! Though I would have preferred being left with my gear.</t>
+  </si>
+  <si>
+    <t>Talked to PC = 0</t>
+  </si>
+  <si>
+    <t>Talked to PC = 0, numMissing &gt;= 4</t>
+  </si>
+  <si>
+    <t>Talked to PC = 0, numMissing &gt; 0</t>
+  </si>
+  <si>
+    <t>Choice "Continue", 1</t>
+  </si>
+  <si>
+    <t>Choice = 1</t>
+  </si>
+  <si>
+    <t>Now then, I expect that you're going to need help leaving?</t>
+  </si>
+  <si>
+    <t>help leaving</t>
+  </si>
+  <si>
+    <t>hasAskedRescue = 0</t>
+  </si>
+  <si>
+    <t>set hasAskedRescue to 1</t>
+  </si>
+  <si>
+    <t>hasAskedRescue = 1, numMissing &gt; 0</t>
+  </si>
+  <si>
+    <t>hasAskedRescue = 1</t>
   </si>
 </sst>
 </file>
@@ -144,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -163,6 +223,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -381,22 +444,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:E1001"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:F1006"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.109375" customWidth="1"/>
     <col min="3" max="3" width="18.88671875" customWidth="1"/>
-    <col min="4" max="4" width="37.6640625" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" customWidth="1"/>
+    <col min="4" max="4" width="37.6640625" style="10" customWidth="1"/>
+    <col min="5" max="5" width="34.109375" customWidth="1"/>
+    <col min="6" max="6" width="31.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -409,8 +473,11 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F3" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
@@ -424,7 +491,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" s="6" customFormat="1" ht="92.4" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
@@ -438,7 +505,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
@@ -452,7 +519,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
@@ -462,8 +529,11 @@
       <c r="D7" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F7" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" s="9" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
@@ -474,92 +544,170 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" s="6" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" s="6" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="B11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" s="6" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="B12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" s="6" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="E15" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" s="6" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="8"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D18" s="1"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D19" s="1"/>
     </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D20" s="1"/>
     </row>
-    <row r="21" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D21" s="1"/>
     </row>
-    <row r="22" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D22" s="1"/>
     </row>
-    <row r="23" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D24" s="1"/>
     </row>
-    <row r="25" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D25" s="1"/>
     </row>
-    <row r="26" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D26" s="1"/>
     </row>
-    <row r="27" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D27" s="1"/>
     </row>
-    <row r="28" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D28" s="1"/>
     </row>
-    <row r="29" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D29" s="1"/>
     </row>
-    <row r="30" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D30" s="1"/>
     </row>
-    <row r="31" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D31" s="1"/>
     </row>
-    <row r="32" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D32" s="1"/>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.25">
@@ -3468,6 +3616,21 @@
     </row>
     <row r="1001" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D1001" s="1"/>
+    </row>
+    <row r="1002" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1002" s="1"/>
+    </row>
+    <row r="1003" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1003" s="1"/>
+    </row>
+    <row r="1004" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1004" s="1"/>
+    </row>
+    <row r="1005" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1005" s="1"/>
+    </row>
+    <row r="1006" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1006" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add: dialogue & script to handle teleporting back
Update: rationalise starting equipment
Update: checks on the rescue ring
</commit_message>
<xml_diff>
--- a/Docs/Dialogue.xlsx
+++ b/Docs/Dialogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAAEA50-D3B7-4ECD-9912-9A1469423918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAFA3C7-DADD-455E-B8B6-11C2D3594EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="47">
   <si>
     <t>Character</t>
   </si>
@@ -143,6 +143,24 @@
   </si>
   <si>
     <t>hasAskedRescue = 1</t>
+  </si>
+  <si>
+    <t>When you're ready to return just let me know. I don't want to send you back without having grabbed everything of value.</t>
+  </si>
+  <si>
+    <t>Choice "I'm ready.", 1, "Hold on, I think there's a place I haven't checked yet.", 2</t>
+  </si>
+  <si>
+    <t>Choice = 2</t>
+  </si>
+  <si>
+    <t>Alrighty then! I'll be right here waiting.</t>
+  </si>
+  <si>
+    <t>StartScript "tlvsos_return" Goodbye</t>
+  </si>
+  <si>
+    <t>Wonderful! I hope you found this little adventure to your liking. Perhaps we shall have another one day, and in the meantime I'll be at your side to love you and care for you with all of my heart.</t>
   </si>
 </sst>
 </file>
@@ -444,7 +462,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:F1006"/>
+  <dimension ref="B1:F1008"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.109375" customWidth="1"/>
@@ -656,58 +674,88 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="2:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="7" t="s">
+    <row r="17" spans="2:6" s="6" customFormat="1" ht="66" x14ac:dyDescent="0.25">
+      <c r="B17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="8"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B19" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D20" s="1"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D21" s="1"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D22" s="1"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D24" s="1"/>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D25" s="1"/>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D26" s="1"/>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D27" s="1"/>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D28" s="1"/>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D29" s="1"/>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D30" s="1"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D31" s="1"/>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D32" s="1"/>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.25">
@@ -3631,6 +3679,12 @@
     </row>
     <row r="1006" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D1006" s="1"/>
+    </row>
+    <row r="1007" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1007" s="1"/>
+    </row>
+    <row r="1008" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1008" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add: fallback line for "place a kiss" topic
Add: MIT License
Update: fill Avatar of Separation's loot chest
</commit_message>
<xml_diff>
--- a/Docs/Dialogue.xlsx
+++ b/Docs/Dialogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\etste\Documents\Projects\Mods\Morrowind\shrine-of-separation\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAFA3C7-DADD-455E-B8B6-11C2D3594EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0004EB0D-83B2-4545-AF3D-855D1C7316F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
   <si>
     <t>Character</t>
   </si>
@@ -121,9 +121,6 @@
     <t>Talked to PC = 0, numMissing &gt; 0</t>
   </si>
   <si>
-    <t>Choice "Continue", 1</t>
-  </si>
-  <si>
     <t>Choice = 1</t>
   </si>
   <si>
@@ -161,6 +158,18 @@
   </si>
   <si>
     <t>Wonderful! I hope you found this little adventure to your liking. Perhaps we shall have another one day, and in the meantime I'll be at your side to love you and care for you with all of my heart.</t>
+  </si>
+  <si>
+    <t>hasSaidValMsg = 1</t>
+  </si>
+  <si>
+    <t>Choice "Continue", 1 set hasSaidValMsg to 1</t>
+  </si>
+  <si>
+    <t>hasSaidValMsg = 0</t>
+  </si>
+  <si>
+    <t>You'd like another peck on the cheek? Or something a bit more involved? Well then, I'm right here my sweet one!</t>
   </si>
 </sst>
 </file>
@@ -462,7 +471,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B1:F1008"/>
+  <dimension ref="B1:F1009"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.109375" customWidth="1"/>
@@ -612,10 +621,10 @@
         <v>17</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
@@ -629,7 +638,7 @@
         <v>29</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="2:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -643,10 +652,10 @@
         <v>28</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" s="6" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
         <v>14</v>
       </c>
@@ -654,13 +663,13 @@
         <v>18</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" s="6" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" s="6" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
         <v>14</v>
       </c>
@@ -668,59 +677,73 @@
         <v>18</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>35</v>
+        <v>19</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" s="6" customFormat="1" ht="66" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" s="6" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" s="6" customFormat="1" ht="66" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D18" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>44</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D19" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="B20" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="D20" s="1"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="D21" s="1"/>
@@ -3685,6 +3708,9 @@
     </row>
     <row r="1008" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D1008" s="1"/>
+    </row>
+    <row r="1009" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1009" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>